<commit_message>
Implement working StudioFlicks scraper with BeautifulSoup
</commit_message>
<xml_diff>
--- a/movies_master.xlsx
+++ b/movies_master.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AK364"/>
+  <dimension ref="A1:AK366"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -44002,6 +44002,192 @@
         </is>
       </c>
     </row>
+    <row r="365">
+      <c r="A365" t="inlineStr">
+        <is>
+          <t>gen__0_hindi</t>
+        </is>
+      </c>
+      <c r="B365" t="inlineStr">
+        <is>
+          <t>_0_hindi</t>
+        </is>
+      </c>
+      <c r="C365" t="inlineStr"/>
+      <c r="D365" t="inlineStr"/>
+      <c r="E365" t="inlineStr">
+        <is>
+          <t>https://www.studioflicks.com/movie/pushpa-2-the-rule/</t>
+        </is>
+      </c>
+      <c r="F365" t="inlineStr">
+        <is>
+          <t>https://img.studioflicks.com/wp-content/uploads/2024/10/17115454/1T21FblunT0y8fz7YaW8JMYgUKm-683x1024.jpg</t>
+        </is>
+      </c>
+      <c r="G365" t="inlineStr"/>
+      <c r="H365" t="n">
+        <v>0</v>
+      </c>
+      <c r="I365" t="inlineStr">
+        <is>
+          <t>Hindi</t>
+        </is>
+      </c>
+      <c r="J365" t="inlineStr"/>
+      <c r="K365" t="inlineStr"/>
+      <c r="L365" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="M365" t="inlineStr"/>
+      <c r="N365" t="inlineStr"/>
+      <c r="O365" t="inlineStr"/>
+      <c r="P365" t="inlineStr"/>
+      <c r="Q365" t="inlineStr"/>
+      <c r="R365" t="inlineStr"/>
+      <c r="S365" t="inlineStr"/>
+      <c r="T365" t="inlineStr"/>
+      <c r="U365" t="inlineStr"/>
+      <c r="V365" t="inlineStr">
+        <is>
+          <t>needs_review</t>
+        </is>
+      </c>
+      <c r="W365" t="inlineStr">
+        <is>
+          <t>new</t>
+        </is>
+      </c>
+      <c r="X365" t="inlineStr">
+        <is>
+          <t>review</t>
+        </is>
+      </c>
+      <c r="Y365" t="b">
+        <v>0</v>
+      </c>
+      <c r="Z365" t="b">
+        <v>0</v>
+      </c>
+      <c r="AA365" t="b">
+        <v>0</v>
+      </c>
+      <c r="AB365" t="inlineStr">
+        <is>
+          <t>2025-12-23T03:45:07.267202</t>
+        </is>
+      </c>
+      <c r="AC365" t="inlineStr">
+        <is>
+          <t>2025-12-23T03:45:07.267212</t>
+        </is>
+      </c>
+      <c r="AD365" t="inlineStr"/>
+      <c r="AE365" t="b">
+        <v>0</v>
+      </c>
+      <c r="AF365" t="inlineStr"/>
+      <c r="AG365" t="inlineStr"/>
+      <c r="AH365" t="inlineStr"/>
+      <c r="AI365" t="inlineStr"/>
+      <c r="AJ365" t="inlineStr"/>
+      <c r="AK365" t="inlineStr"/>
+    </row>
+    <row r="366">
+      <c r="A366" t="inlineStr">
+        <is>
+          <t>gen__0_hindi</t>
+        </is>
+      </c>
+      <c r="B366" t="inlineStr">
+        <is>
+          <t>_0_hindi</t>
+        </is>
+      </c>
+      <c r="C366" t="inlineStr"/>
+      <c r="D366" t="inlineStr"/>
+      <c r="E366" t="inlineStr">
+        <is>
+          <t>https://www.studioflicks.com/movie/game-changer/</t>
+        </is>
+      </c>
+      <c r="F366" t="inlineStr">
+        <is>
+          <t>https://img.studioflicks.com/wp-content/uploads/2025/01/13123419/Game-Changer-Movie-HD-Poster-9-683x1024.jpg</t>
+        </is>
+      </c>
+      <c r="G366" t="inlineStr"/>
+      <c r="H366" t="n">
+        <v>0</v>
+      </c>
+      <c r="I366" t="inlineStr">
+        <is>
+          <t>Hindi</t>
+        </is>
+      </c>
+      <c r="J366" t="inlineStr"/>
+      <c r="K366" t="inlineStr"/>
+      <c r="L366" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="M366" t="inlineStr"/>
+      <c r="N366" t="inlineStr"/>
+      <c r="O366" t="inlineStr"/>
+      <c r="P366" t="inlineStr"/>
+      <c r="Q366" t="inlineStr"/>
+      <c r="R366" t="inlineStr"/>
+      <c r="S366" t="inlineStr"/>
+      <c r="T366" t="inlineStr"/>
+      <c r="U366" t="inlineStr"/>
+      <c r="V366" t="inlineStr">
+        <is>
+          <t>needs_review</t>
+        </is>
+      </c>
+      <c r="W366" t="inlineStr">
+        <is>
+          <t>new</t>
+        </is>
+      </c>
+      <c r="X366" t="inlineStr">
+        <is>
+          <t>review</t>
+        </is>
+      </c>
+      <c r="Y366" t="b">
+        <v>0</v>
+      </c>
+      <c r="Z366" t="b">
+        <v>0</v>
+      </c>
+      <c r="AA366" t="b">
+        <v>0</v>
+      </c>
+      <c r="AB366" t="inlineStr">
+        <is>
+          <t>2025-12-23T03:45:10.579290</t>
+        </is>
+      </c>
+      <c r="AC366" t="inlineStr">
+        <is>
+          <t>2025-12-23T03:45:10.579304</t>
+        </is>
+      </c>
+      <c r="AD366" t="inlineStr"/>
+      <c r="AE366" t="b">
+        <v>0</v>
+      </c>
+      <c r="AF366" t="inlineStr"/>
+      <c r="AG366" t="inlineStr"/>
+      <c r="AH366" t="inlineStr"/>
+      <c r="AI366" t="inlineStr"/>
+      <c r="AJ366" t="inlineStr"/>
+      <c r="AK366" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>